<commit_message>
Update documents: modified and removed files
</commit_message>
<xml_diff>
--- a/Задача від 14.10.2026 переклад французька/1. Общие справки и систематизация материалов/20260813 Registre des pieces du dossier affaire francaise.xlsx
+++ b/Задача від 14.10.2026 переклад французька/1. Общие справки и систематизация материалов/20260813 Registre des pieces du dossier affaire francaise.xlsx
@@ -1359,7 +1359,7 @@
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>Monaco ; résidence fiscale / statut de résident ; véhicules ; Laterson ; Monacuiros</t>
+          <t>Monaco ; résidence ; véhicules ; Laterson ; Monacuiros</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -1468,7 +1468,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Réponse de Maître Luciani, notaire, à la réquisition judiciaire portant sur l'origine des fonds utilisés pour les acquisitions immobilières par les SCI Slava, Belle Époque, Promenade des Anglais, Des Anges et Saint Petr.</t>
+          <t>Réponse du notaire Luciani à la réquisition judiciaire sur l'origine des fonds en lien avec l'achat-vente des SCI Slava, Belle Epoque, Promenade Des Anglais, Des Anges, Saint Petr.</t>
         </is>
       </c>
     </row>
@@ -2143,7 +2143,7 @@
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>Monaco ; AVB ; résidence fiscale / statut de résident</t>
+          <t>Monaco ; AVB ; résidence</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
@@ -2792,7 +2792,7 @@
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>Information relative à la saisie pénale conservatoire des fonds d'un montant de 1 035 000 EUR séquestrés sur le compte de l'étude notariale de Maître Dogliani, issus de la vente de l'actif immobilier de la SCI Des Anges.</t>
+          <t>Information relative à la saisie des fonds (1,035 M EUR) sur le compte du notaire Dogliani, provenant de la vente de la SCI Des Anges.</t>
         </is>
       </c>
     </row>
@@ -4848,7 +4848,7 @@
       </c>
       <c r="F164" s="3" t="inlineStr">
         <is>
-          <t>Procès-verbal d'examen du compte bancaire ouvert au nom de VAB à La Banque Postale. Relève le dossier d'ouverture de compte, les pièces d'identité ukrainiennes, la carte de résident monégasque, une attestation établie par Motor Bank, la déclaration de résidence au One Monte-Carlo, la procuration bancaire accordée par AVB sur le compte de son père et l'analyse de la nature des débits.</t>
+          <t>Procès-verbal d'examen du compte bancaire ouvert au nom de VAB à La Banque Postale. Sont consignés les documents d'ouverture de compte, les documents ukrainiens, la carte de résident de Monaco, une attestation de Motor Bank, la résidence au One Monte-Carlo, la procuration d'AVB sur le compte de son fils [Note : l'original mentionne à la fois le compte de VAB et « la procuration d'AVB sur le compte du fils »] et la nature des dépenses.</t>
         </is>
       </c>
     </row>
@@ -5616,7 +5616,7 @@
       </c>
       <c r="F188" s="3" t="inlineStr">
         <is>
-          <t>Procès-verbal constatant l'émission d'une demande urgente de levée du principe de spécialité consécutive à l'exécution de l'entraide judiciaire à Monaco. Sont joints la requête du parquet français, la convention portant création de l'équipe commune d'enquête (ÉCI / JIT) franco-ukrainienne et l'inventaire des scellés saisis lors des perquisitions à Monaco.</t>
+          <t>Procès-verbal de réception d'une demande urgente de levée du principe de spécialité consécutive à l'exécution de l'entraide judiciaire à Monaco. Sont joints la requête du parquet français, la convention portant création de l'équipe commune d'enquête (ÉCI / JIT) franco-ukrainienne et l'inventaire des scellés saisis lors des perquisitions à Monaco.</t>
         </is>
       </c>
     </row>
@@ -9448,7 +9448,7 @@
       </c>
       <c r="F308" s="7" t="inlineStr">
         <is>
-          <t>Procès-verbal relatif aux relations d'intérêts et liens de détention entre la société Katran Ltd et M. Vnukov.</t>
+          <t>Procès-verbal relatif aux liens entre la société Katran LTD et M. Vnukov.</t>
         </is>
       </c>
     </row>
@@ -10088,7 +10088,7 @@
       </c>
       <c r="F328" s="7" t="inlineStr">
         <is>
-          <t>Procès-verbal d'examen de l'avenant du 19/12/2014 au protocole d'accord du 17/05/2014 signé par Wang Jing. L'acte énonce explicitement l'accord des parties dispensant l'acquisition d'actions de toute autorisation de concentration auprès de l'AMKU (Comité anti-monopole d'Ukraine), clause jugée équivoque par les enquêteurs au regard du respect de la réglementation anti-monopole.</t>
+          <t>Procès-verbal d'examen de l'Amendment Agreement du 19/12/2014 au MOU du 17/05/2014 signé par Wang Jing. Le document contient explicitement une disposition selon laquelle les parties confirment qu'une autorisation de concentration de l'AMKU (Comité anti-monopole d'Ukraine) n'est pas nécessaire pour l'acquisition d'actions concernée. L'enquête considère cette disposition comme soulevant une question quant au respect des exigences anti-monopole.</t>
         </is>
       </c>
     </row>
@@ -10280,7 +10280,7 @@
       </c>
       <c r="F334" s="7" t="inlineStr">
         <is>
-          <t>Procès-verbal d'examen de la correspondance du 24/02/2015 entre M. Katsylo et AVB relative aux risques entourant le « Project Zoom » : nécessité d'extraire Motor Bank du périmètre contractuel, son maintien risquant de susciter une forte médiatisation de l'opération, des risques d'annulation judiciaire et des sanctions politiques ; analyse de l'acquisition des titres de MS sans agrément préalable de l'AMKU et options de cession de Motor Bank avant ou après la finalisation.</t>
+          <t>Procès-verbal d'examen de la correspondance du 24/02/2015 entre M. Katsylo et AVB sur les risques liés au « Project Zoom ». Est discutée la nécessité d'exclure Motor Bank du périmètre de la transaction, car son inclusion pourrait entraîner la publicité de la transaction, des conséquences politiques et juridiques ainsi qu'un risque de contestation/nullité de celle-ci. La question de l'acquisition des actions de MS sans autorisation préalable de l'AMKU est posée séparément et des options de sortie de Motor Bank avant ou après la clôture de la transaction sont proposées.</t>
         </is>
       </c>
     </row>
@@ -13526,7 +13526,7 @@
       </c>
       <c r="D438" s="7" t="inlineStr">
         <is>
-          <t>Résidence fiscale ; Revenus</t>
+          <t>Résidence ; Revenus</t>
         </is>
       </c>
       <c r="E438" s="7" t="inlineStr">
@@ -13751,7 +13751,7 @@
       </c>
       <c r="E445" s="7" t="inlineStr">
         <is>
-          <t>AVB ; auditions ; Monaco ; actifs ; revenus ; sociétés offshore ; MS ; ME ; résidence fiscale</t>
+          <t>AVB ; auditions ; Monaco ; actifs ; revenus ; sociétés offshore ; MS ; ME ; résidence</t>
         </is>
       </c>
       <c r="F445" s="7" t="inlineStr">
@@ -13778,7 +13778,7 @@
       </c>
       <c r="D446" s="7" t="inlineStr">
         <is>
-          <t>Auditions / Actifs / Revenus / Sociétés offshore / Résidence fiscale</t>
+          <t>Auditions / Actifs / Revenus / Sociétés offshore / Résidence</t>
         </is>
       </c>
       <c r="E446" s="7" t="inlineStr">
@@ -15090,7 +15090,7 @@
       </c>
       <c r="D488" s="7" t="inlineStr">
         <is>
-          <t>Téléphonie ; Actifs ; Résidence fiscale</t>
+          <t>Téléphone ; Actifs ; Résidence</t>
         </is>
       </c>
       <c r="E488" s="7" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="F488" s="7" t="inlineStr">
         <is>
-          <t>Procès-verbal d'exploitation technique par l'ONAF du téléphone portable d'AVB : relevés de géolocalisation, messageries WhatsApp et Telegram, documents de bail locatif, TLC Group, résidence fiscale monégasque, véhicules et patrimoine.</t>
+          <t>Procès-verbal d'exploitation technique par l'ONAF du téléphone portable d'AVB : relevés de géolocalisation, messageries WhatsApp et Telegram, documents de bail locatif, TLC Group, résidence à Monaco, véhicules et patrimoine.</t>
         </is>
       </c>
     </row>
@@ -15122,7 +15122,7 @@
       </c>
       <c r="D489" s="7" t="inlineStr">
         <is>
-          <t>Résidence fiscale ; Actifs</t>
+          <t>Résidence ; Actifs</t>
         </is>
       </c>
       <c r="E489" s="7" t="inlineStr">
@@ -15144,7 +15144,7 @@
       </c>
       <c r="B490" s="7" t="inlineStr">
         <is>
-          <t>EXH_T4_PV163_02_Facture_TLC_Group_residence_fiscale_Monaco</t>
+          <t>EXH_T4_PV163_02_Facture_TLC_Group_residence_Monaco</t>
         </is>
       </c>
       <c r="C490" s="7" t="inlineStr">
@@ -15159,12 +15159,12 @@
       </c>
       <c r="E490" s="7" t="inlineStr">
         <is>
-          <t>TLC Group ; AVB ; Monaco ; résidence fiscale</t>
+          <t>TLC Group ; AVB ; Monaco ; résidence</t>
         </is>
       </c>
       <c r="F490" s="7" t="inlineStr">
         <is>
-          <t>Facture de la société TLC Group du 4 février 2025 d'un montant de 18 000 EUR au titre de l'audit de conformité d'AVB aux critères de résidence fiscale à Monaco pour la période 2015-2024.</t>
+          <t>Facture de TLC Group du 04/02/2025 d'un montant de 18 000 EUR pour l'analyse des obligations d'AVB relatives au respect des critères de résidence à Monaco pour la période 2015–2024.</t>
         </is>
       </c>
     </row>
@@ -15176,7 +15176,7 @@
       </c>
       <c r="B491" s="7" t="inlineStr">
         <is>
-          <t>EXH_T4_PV163_03_Rapport_TLC_Group_residence_fiscale_Monaco</t>
+          <t>EXH_T4_PV163_03_Rapport_TLC_Group_residence_Monaco</t>
         </is>
       </c>
       <c r="C491" s="7" t="inlineStr">
@@ -15191,12 +15191,12 @@
       </c>
       <c r="E491" s="7" t="inlineStr">
         <is>
-          <t>TLC Group ; AVB ; Monaco ; résidence fiscale</t>
+          <t>TLC Group ; AVB ; Monaco ; résidence</t>
         </is>
       </c>
       <c r="F491" s="7" t="inlineStr">
         <is>
-          <t>Rapport d'analyse pluriannuel établi par TLC Group attestant de la résidence fiscale effective d'AVB à Monaco.</t>
+          <t>Analyse de TLC Group par année, liée à la confirmation de la résidence d'AVB à Monaco.</t>
         </is>
       </c>
     </row>
@@ -15236,7 +15236,7 @@
       </c>
       <c r="B493" s="7" t="inlineStr">
         <is>
-          <t>T4_PGS_PV165_Analyse_rapport_TLC_Group_residence_fiscale_AVB_Monaco</t>
+          <t>T4_PGS_PV165_Analyse_rapport_TLC_Group_residence_AVB_Monaco</t>
         </is>
       </c>
       <c r="C493" s="7" t="inlineStr">

</xml_diff>

<commit_message>
Update repository files and documents
</commit_message>
<xml_diff>
--- a/Задача від 14.10.2026 переклад французька/1. Общие справки и систематизация материалов/20260813 Registre des pieces du dossier affaire francaise.xlsx
+++ b/Задача від 14.10.2026 переклад французька/1. Общие справки и систематизация материалов/20260813 Registre des pieces du dossier affaire francaise.xlsx
@@ -532,7 +532,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Réquisition judiciaire et note de renseignement en réponse de TRACFIN concernant AVB (Anton Boguslayev), VAB (Vyacheslav Boguslayev), les SCI Belle Époque, Promenade des Anglais, Des Anges, Saint Petr, Kozak, Aviwell 3000, Vera, etc.</t>
+          <t>Réquisition judiciaire et note de renseignement en réponse de TRACFIN concernant AVB (Oleksandr Boguslayev), VAB (Vyacheslav Boguslayev), les SCI Belle Époque, Promenade des Anglais, Des Anges, Saint Petr, Kozak, Aviwell 3000, Vera, etc.</t>
         </is>
       </c>
     </row>
@@ -552,7 +552,7 @@
       <c r="E4" s="2" t="n"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Note de renseignement en réponse de TRACFIN à la réquisition judiciaire concernant AVB (Anton Boguslayev), VAB (Vyacheslav Boguslayev), les SCI Belle Époque, Promenade des Anglais, Des Anges, Saint Petr, Kozak, Aviwell 3000, Vera, etc.</t>
+          <t>Note de renseignement en réponse de TRACFIN à la réquisition judiciaire concernant AVB (Oleksandr Boguslayev), VAB (Vyacheslav Boguslayev), les SCI Belle Époque, Promenade des Anglais, Des Anges, Saint Petr, Kozak, Aviwell 3000, Vera, etc.</t>
         </is>
       </c>
     </row>
@@ -1580,7 +1580,7 @@
       <c r="E41" s="3" t="n"/>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>Acte authentique de vente immobilière du chalet « Le Petit Vah » situé à Courchevel en date du 14 octobre 2019, conclu entre la SCI Foehn Bellecôte et Monacourch pour un montant de 4 250 000 EUR.</t>
+          <t>Acte de vente immobilière du chalet « Le Petit Vah » à Courchevel en date du 14 octobre 2019 conclu entre la SCI Foehn Bellecôte et Monacourch (SPA).</t>
         </is>
       </c>
     </row>
@@ -1704,7 +1704,7 @@
       <c r="E47" s="3" t="n"/>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>Acte authentique de vente immobilière conclu le 16 janvier 2020 entre la SCI Vera et NH Appart portant sur un appartement sis 2, rue Guiglia, 06000 Nice, pour un montant de 1 050 000 EUR.</t>
+          <t>Acte de vente immobilière conclu entre la SCI Vera et NH Appart portant sur un appartement sis 2, rue Guiglia, 06000 Nice, EUR 1 050 000.</t>
         </is>
       </c>
     </row>
@@ -2292,7 +2292,7 @@
       <c r="A71" s="2" t="n"/>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>EXH_T2_PV039_2_SPA_27.03.2017_SCI_Kozak_EUR10,650M_12av_Prince_Rainier_III_SJCF</t>
+          <t>EXH_T2_PV039_2_SPA 27.07.2017 by SCI Kozak EUR10,650 _12av Prince Rainier III, SJCF</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
@@ -2304,7 +2304,7 @@
       <c r="E71" s="2" t="n"/>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>Acte authentique de vente immobilière du bien sis 12, avenue Prince Rainier III en date du 27 mars 2017.</t>
+          <t>Acte de vente immobilière du bien sis 12, avenue Prince Rainier III en date du 27 mars 2017 [Note : l'identifiant en colonne B mentionne 27.07.2017].</t>
         </is>
       </c>
     </row>
@@ -3835,12 +3835,12 @@
       </c>
       <c r="E131" s="2" t="inlineStr">
         <is>
-          <t>JSC « Motor Sich » (ci-après « MS ») ; perquisitions Monaco ; AVB (Anton Vyacheslavovych Boguslayev / Anton Boguslayev)</t>
+          <t>JSC « Motor Sich » (ci-après « MS ») ; perquisitions Monaco ; AVB (Oleksandr Vyacheslavovych Boguslayev / Oleksandr Boguslayev)</t>
         </is>
       </c>
       <c r="F131" s="2" t="inlineStr">
         <is>
-          <t>Documents saisis lors des perquisitions des coffres-forts bancaires d'AVB (Anton Vyacheslavovych Boguslayev / Anton Boguslayev) à Monaco : listes d'entités sociétaires non-résidentes et schémas / organigrammes de structures offshore (Chypre, Belize, Îles Vierges britanniques / BVI, Panama, etc.).</t>
+          <t>Documents saisis lors des perquisitions des coffres-forts bancaires d'AVB (Oleksandr Vyacheslavovych Boguslayev / Oleksandr Boguslayev) à Monaco : listes d'entités sociétaires non-résidentes et schémas / organigrammes de structures offshore (Chypre, Belize, Îles Vierges britanniques / BVI, Panama, etc.).</t>
         </is>
       </c>
     </row>
@@ -3887,7 +3887,7 @@
       </c>
       <c r="E133" s="2" t="inlineStr">
         <is>
-          <t>Escrow ; perquisitions Monaco ; AVB (Anton Vyacheslavovych Boguslayev / Anton Boguslayev)</t>
+          <t>Escrow ; perquisitions Monaco ; AVB (Oleksandr Vyacheslavovych Boguslayev / Oleksandr Boguslayev)</t>
         </is>
       </c>
       <c r="F133" s="2" t="inlineStr">
@@ -3988,7 +3988,7 @@
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>Description des pièces saisies lors des perquisitions des coffres bancaires d'AVB à Monaco : original du contrat de bail du studio Château Périgord à Monaco (24 000 EUR par an) ; original du contrat de bail de l'appartement sis Villa Gaston-Suzanne, 7 rue Révérend Père Louis Frolla à Monaco (36 000 EUR par an) ; original du contrat de bail du triplex situé One Monte-Carlo, Place du Casino, C (2 600 000 EUR par an). Montant cumulé des loyers : 10 460 000 EUR sur la période.</t>
+          <t>Description des pièces saisies lors des perquisitions des coffres bancaires d'AVB à Monaco : original du contrat de bail du studio Château Périgord à Monaco (24 000 EUR par an) ; original du contrat de bail de l'appartement sis Villa Gaston-Suzanne, 7 rue Révérend Père Louis Frolla à Monaco (36 000 EUR par an) ; original du contrat de bail du triplex situé One Monte-Carlo, Place du Casino, C (2 600 000 EUR par an). Montant total des loyers : 10,46 millions EUR par an [sic ; la somme arithmétique des trois loyers annuels s'élève à 2 660 000 EUR par an].</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>Description des pièces saisies lors des perquisitions des coffres bancaires d'AVB à Monaco : documents originaux relatifs à l'acquisition de la propriété « La Petite Afrique » par la société Laterson pour un montant de 60 000 000 EUR ; lettre d'AVB en date du 06/10/2015 constatant l'impossibilité de s'acquitter de 28 000 000 EUR ; lettre d'AVB en date du 12/01/2016 reconnaissant l'obligation de verser des intérêts moratoires pour retard de paiement ; confirmation d'un virement bancaire d'un montant de 218 647,28 EUR ; compromis de vente du 24/06/2015 ; quittance de l'étude notariale Aureglia-Caruso constatant la réception de 6 000 000 EUR en provenance de la banque BPS de la part d'AVB ; quittance notariale constatant la réception de 20 000 000 EUR de la société Laterson, etc.</t>
+          <t>Description des pièces saisies lors des perquisitions des coffres bancaires d'AVB à Monaco : documents originaux relatifs à l'acquisition de la propriété « La Petite Afrique » par la société Laterson pour un montant de 60 000 000 EUR ; lettre d'AVB en date du 6 octobre 2015 constatant l'impossibilité de s'acquitter de 28 000 000 EUR ; lettre d'AVB en date du 12 janvier 2016 reconnaissant l'obligation de verser des intérêts moratoires pour retard de paiement ; confirmation d'un virement bancaire d'un montant de 218 647,28 EUR ; compromis de vente du 24 juin 2015 ; quittance de l'étude notariale Aureglia-Caruso constatant la réception de 6 000 000 EUR en provenance de la banque BPS de la part d'AVB ; quittance notariale constatant la réception de 20 000 000 EUR de la société Laterson, etc.</t>
         </is>
       </c>
     </row>
@@ -5040,7 +5040,7 @@
       </c>
       <c r="F170" s="3" t="inlineStr">
         <is>
-          <t>Procès-verbal de notification de l'ordonnance du juge d'instruction en date du 19/09/2023 ordonnant la saisie pénale conservatoire de parts sociales au sein des SCI.</t>
+          <t>Procès-verbal de notification de l'ordonnance du juge d'instruction en date du 19 septembre 2023 ordonnant la saisie pénale conservatoire de parts sociales au sein des SCI.</t>
         </is>
       </c>
     </row>
@@ -5200,7 +5200,7 @@
       </c>
       <c r="F175" s="3" t="inlineStr">
         <is>
-          <t>Procès-verbal de réception de l'ordonnance du Juge des libertés et de la détention (JLD) en date du 21/10/2023 autorisant des opérations de perquisition, visite domiciliaire et saisie de pièces à conviction et supports numériques sans l'assentiment de la personne (visant notamment les sites de Saint-Jean-Cap-Ferrat et du Domaine de Cuiros).</t>
+          <t>Procès-verbal de réception de l'ordonnance du Juge des libertés et de la détention (JLD) en date du 21 octobre 2023 autorisant des opérations de perquisition, visite domiciliaire et saisie de pièces à conviction et supports numériques sans l'assentiment de la personne (visant notamment les sites de Saint-Jean-Cap-Ferrat et du Domaine de Cuiros).</t>
         </is>
       </c>
     </row>
@@ -5296,7 +5296,7 @@
       </c>
       <c r="F178" s="3" t="inlineStr">
         <is>
-          <t>Procès-verbal de réception et de prise en charge des scellés et pièces à conviction transmis par la police de Monaco, saisis lors des perquisitions des coffres bancaires d'AVB chez Julius Baer et UBP les 18 et 19/10/2023 (documentation relative aux sociétés offshore, SCI, Fraser, Laterson, etc.).</t>
+          <t>Procès-verbal de réception et de prise en charge des scellés et pièces à conviction transmis par la police de Monaco, saisis lors des perquisitions des coffres bancaires d'AVB chez Julius Baer et UBP les 18 et 19 octobre 2023 (documentation relative aux sociétés offshore, SCI, Fraser, Laterson, etc.).</t>
         </is>
       </c>
     </row>
@@ -5328,7 +5328,7 @@
       </c>
       <c r="F179" s="3" t="inlineStr">
         <is>
-          <t>Procès-verbal de dépôt sécurisé auprès de la société Loomis du scellé monétaire comprenant 10 650 CHF en espèces saisis dans le coffre-fort d'AVB à la banque UBP Monaco.</t>
+          <t>Procès-verbal de remise en dépôt de scellés (pièces à conviction) saisis dans le coffre-fort d'AVB auprès d'UBP.</t>
         </is>
       </c>
     </row>
@@ -5392,7 +5392,7 @@
       </c>
       <c r="F181" s="3" t="inlineStr">
         <is>
-          <t>Procès-verbal de réception de renseignements complémentaires transmis le 05/12/2023 par le Bureau du Procureur général d'Ukraine (OGP) dans le cadre de l'entraide judiciaire internationale en matière pénale.</t>
+          <t>Procès-verbal de réception de renseignements complémentaires transmis le 5 décembre 2023 par le Bureau du Procureur général d'Ukraine (OGP) dans le cadre de l'entraide judiciaire internationale en matière pénale.</t>
         </is>
       </c>
     </row>
@@ -5424,7 +5424,7 @@
       </c>
       <c r="F182" s="3" t="inlineStr">
         <is>
-          <t>Procès-verbal d'analyse des informations complémentaires transmises par les autorités ukrainiennes le 05/12/2023 : porte sur les revenus perçus par VAB et AVB, la cession d'actions de MS, la structuration des circuits financiers et les intermédiaires bancaires (Likatron, Skyrizon, UBI Banca, Motor Bank).</t>
+          <t>Procès-verbal d'analyse des informations complémentaires transmises par les autorités ukrainiennes le 5 décembre 2023 : porte sur les revenus perçus par VAB et AVB, la cession d'actions de MS, la structuration des circuits financiers et les intermédiaires bancaires (Likatron, Skyrizon, UBI Banca, Motor Bank).</t>
         </is>
       </c>
     </row>
@@ -5456,7 +5456,7 @@
       </c>
       <c r="F183" s="3" t="inlineStr">
         <is>
-          <t>Procès-verbal de recoupement entre les informations complémentaires ukrainiennes du 05/12/2023 et les pièces saisies dans les coffres-forts d'AVB à Monaco : corrélation des sociétés offshore (Business House Helena, Enfields, Skyrizon, Laterson) et de l'acquisition de la SCI Carré d'Or Quadruplex.</t>
+          <t>Procès-verbal de recoupement entre les informations complémentaires ukrainiennes du 5 décembre 2023 et les pièces saisies dans les coffres-forts d'AVB à Monaco : corrélation des sociétés offshore (Business House Helena, Enfields, Skyrizon, Laterson) et de l'acquisition de la SCI Carré d'Or Quadruplex.</t>
         </is>
       </c>
     </row>
@@ -5488,7 +5488,7 @@
       </c>
       <c r="F184" s="3" t="inlineStr">
         <is>
-          <t>Procès-verbal de rapprochement entre les revenus déclarés et le train de vie d'AVB : les enquêteurs soulignent la disproportion manifeste entre un revenu déclaré en 2016 en Ukraine (initialement évalué à tort à environ 390 000 000 UAH, rectifié ensuite à 390 000 UAH) et l'acquisition / jouissance de biens somptuaires en France, à Monaco, à Dubaï et au Monténégro (yachts Slava et Kozak, triplex au One Monte-Carlo, actifs immobiliers de prestige).</t>
+          <t>Procès-verbal de rapprochement des revenus et du train de vie d'AVB. L'enquête fait état d'un revenu d'AVB pour l'année 2016 d'environ 390 millions UAH [Note : rectifié ultérieurement comme erreur matérielle à 390 000 UAH dans le PV du 27 mars 2024, voir ligne 205], de revenus antérieurs nettement inférieurs, ainsi que de l'acquisition / utilisation d'actifs en France, à Monaco, à Dubaï et au Monténégro.</t>
         </is>
       </c>
     </row>
@@ -5712,7 +5712,7 @@
       </c>
       <c r="F191" s="7" t="inlineStr">
         <is>
-          <t>Procès-verbal de réception de la décision de la Direction des Services Judiciaires de la Principauté de Monaco accordant formellement la levée du principe de spécialité sur les scellés saisis les 18 et 19/10/2023.</t>
+          <t>Procès-verbal de réception de la décision de la Direction des Services Judiciaires de la Principauté de Monaco accordant formellement la levée du principe de spécialité sur les scellés saisis les 18 et 19 octobre 2023.</t>
         </is>
       </c>
     </row>
@@ -5776,7 +5776,7 @@
       </c>
       <c r="F193" s="3" t="inlineStr">
         <is>
-          <t>Procès-verbal constatant l'exploitation conjointe par la France et l'Ukraine des pièces et scellés saisis à Monaco les 18 et 19/10/2023 : détaille les perquisitions des coffres d'AVB à Monaco, la remise des scellés aux enquêteurs français, l'institution de l'ÉCI, la levée du principe de spécialité et la mise à disposition de la délégation ukrainienne des copies conformes des supports numériques.</t>
+          <t>Procès-verbal constatant l'exploitation conjointe par la France et l'Ukraine des pièces et scellés saisis à Monaco les 18 et 19 octobre 2023 : détaille les perquisitions des coffres d'AVB à Monaco, la remise des scellés aux enquêteurs français, l'institution de l'ÉCI, la levée du principe de spécialité et la mise à disposition de la délégation ukrainienne des copies conformes des supports numériques.</t>
         </is>
       </c>
     </row>
@@ -5872,7 +5872,7 @@
       </c>
       <c r="F196" s="3" t="inlineStr">
         <is>
-          <t>Procès-verbal consignant les renseignements exposés au cours de la réunion de travail tenue du 19 au 23/02/2024 avec les enquêteurs ukrainiens : expose la thèse de l'accusation ukrainienne à l'encontre de VAB, de Pavlo Zaruba et d'Oleg Zaruba (livraisons triangulaires via la Chine et les Émirats arabes unis, violation de l'embargo, rôle central de MS).</t>
+          <t>Procès-verbal consignant les renseignements exposés au cours de la réunion de travail tenue du 19 au 23 février 2024 avec les enquêteurs ukrainiens : expose la thèse de l'accusation ukrainienne à l'encontre de VAB, de Pavlo Zaruba et d'Oleg Zaruba (livraisons triangulaires via la Chine et les Émirats arabes unis, violation de l'embargo, rôle central de MS).</t>
         </is>
       </c>
     </row>
@@ -5904,7 +5904,7 @@
       </c>
       <c r="F197" s="7" t="inlineStr">
         <is>
-          <t>Procès-verbal d'exploitation forensique de l'ordinateur d'AVB saisi à Monaco : découverte de titres de transport aérien Austrian Airlines et de réservations hôtelières Booking.com matérialisant la présence d'AVB au Luxembourg du 15 au 18/05/2015.</t>
+          <t>Procès-verbal d'exploitation forensique de l'ordinateur d'AVB saisi à Monaco : découverte de titres de transport aérien Austrian Airlines et de réservations hôtelières Booking.com matérialisant la présence d'AVB au Luxembourg du 15 au 18 mai 2015.</t>
         </is>
       </c>
     </row>
@@ -5968,7 +5968,7 @@
       </c>
       <c r="F199" s="3" t="inlineStr">
         <is>
-          <t>Procès-verbal de réception et d'analyse de la réponse délivrée par la Suisse au titre de l'entraide judiciaire : constatation du virement de 824 868,88 USD intervenu le 27/05/2022 vers le compte bancaire de VAB chez Motor Bank, suivi de la clôture définitive du compte suisse le 30/05/2022.</t>
+          <t>Procès-verbal de réception et d'analyse de la réponse délivrée par la Suisse au titre de l'entraide judiciaire : constatation du virement de 824 868,88 USD intervenu le 27 mai 2022 vers le compte bancaire de VAB chez Motor Bank, suivi de la clôture définitive du compte suisse le 30 mai 2022.</t>
         </is>
       </c>
     </row>
@@ -6000,7 +6000,7 @@
       </c>
       <c r="F200" s="3" t="inlineStr">
         <is>
-          <t>Procès-verbal de constatation en ligne d'un article du quotidien Financial Times en date du 11/03/2021 relatif à la nationalisation de MS par les autorités ukrainiennes pour faire échec à la prise de contrôle par des entités chinoises.</t>
+          <t>Procès-verbal de constatation en ligne d'un article du quotidien Financial Times en date du 11 mars 2021 relatif à la nationalisation de MS par les autorités ukrainiennes pour faire échec à la prise de contrôle par des entités chinoises.</t>
         </is>
       </c>
     </row>
@@ -6128,7 +6128,7 @@
       </c>
       <c r="F204" s="3" t="inlineStr">
         <is>
-          <t>Procès-verbal de réception et d'analyse des pièces complémentaires ukrainiennes des 06/12/2023 et 04/01/2024 : expose les données de revenus de VAB, la cession d'actions de MS, l'encaissement de 43 000 000 USD versés par Likatron Enterprises Limited / Wang Xinlei, le circuit financier via China Development Bank, UBI Banca Luxembourg et Motor Bank, ainsi que la cartographie des comptes chez UBI Banca et les éléments relatifs à Skyrizon sous le régime des sanctions.</t>
+          <t>Procès-verbal de réception et d'analyse des pièces complémentaires ukrainiennes des 6 décembre 2023 et 4 janvier 2024 : expose les données de revenus de VAB, la cession d'actions de MS, l'encaissement de 43 000 000 USD versés par Likatron Enterprises Limited / Wang Xinlei, le circuit financier via China Development Bank, UBI Banca Luxembourg et Motor Bank, ainsi que la cartographie des comptes chez UBI Banca et les éléments relatifs à Skyrizon sous le régime des sanctions.</t>
         </is>
       </c>
     </row>
@@ -6160,7 +6160,7 @@
       </c>
       <c r="F205" s="3" t="inlineStr">
         <is>
-          <t>Procès-verbal d'analyse des informations complémentaires transmises par l'Ukraine le 27/03/2024 : traite de la procédure d'arbitrage international engagée par les actionnaires chinois de MS contre l'Ukraine devant la Cour permanente d'arbitrage (CPA) de La Haye, de l'autorisation donnée par le ministère de la Justice d'Ukraine pour transmettre les pièces à la France et à Monaco, de la requête tendant à l'exploitation des pièces de l'ÉCI pour la défense de l'Ukraine dans l'arbitrage, et rectifie l'erreur matérielle relative aux revenus perçus par AVB en 2016 (390 000 UAH et non 390 000 000 UAH).</t>
+          <t>Procès-verbal d'analyse des informations complémentaires transmises par l'Ukraine le 27 mars 2024 : traite de la procédure d'arbitrage international engagée par les actionnaires chinois de MS contre l'Ukraine devant la Cour permanente d'arbitrage (CPA) de La Haye, de l'autorisation donnée par le ministère de la Justice d'Ukraine pour transmettre les pièces à la France et à Monaco, de la requête tendant à l'exploitation des pièces de l'ÉCI pour la défense de l'Ukraine dans l'arbitrage, et rectifie l'erreur matérielle relative aux revenus perçus par AVB en 2016 (390 000 UAH et non 390 000 000 UAH).</t>
         </is>
       </c>
     </row>
@@ -6192,7 +6192,7 @@
       </c>
       <c r="F206" s="3" t="inlineStr">
         <is>
-          <t>Procès-verbal de réquisition délivrée à la compagnie Austrian Airlines et analyse des historiques de vols effectués par AVB depuis le 01/01/2022 : relève des déplacements sur les lignes Vienne / Nice / Podgorica / Innsbruck et diverses données de voyage.</t>
+          <t>Procès-verbal de réquisition délivrée à la compagnie Austrian Airlines et analyse des historiques de vols effectués par AVB depuis le 1er janvier 2022 : relève des déplacements sur les lignes Vienne / Nice / Podgorica / Innsbruck et diverses données de voyage.</t>
         </is>
       </c>
     </row>
@@ -6224,7 +6224,7 @@
       </c>
       <c r="F207" s="3" t="inlineStr">
         <is>
-          <t>Procès-verbal d'examen du dossier administratif d'AVB auprès des autorités monégasques (demandes et renouvellements de cartes de séjour / résident) : situation d'état civil, nationalités ukrainienne et de la Grenade, résidence à Monaco attestée depuis le 08/10/2015, adresses successives, One Monte-Carlo, contrats de bail, présence supérieure à 183 jours par an, absence d'antécédents défavorables et déclarations de patrimoine.</t>
+          <t>Procès-verbal d'examen du dossier administratif d'AVB auprès des autorités monégasques (demandes et renouvellements de cartes de séjour / résident) : situation d'état civil, nationalités ukrainienne et de la Grenade, résidence à Monaco attestée depuis le 8 octobre 2015, adresses successives, One Monte-Carlo, contrats de bail, présence supérieure à 183 jours par an, absence d'antécédents défavorables et déclarations de patrimoine.</t>
         </is>
       </c>
     </row>
@@ -6544,7 +6544,7 @@
       </c>
       <c r="F217" s="3" t="inlineStr">
         <is>
-          <t>Procès-verbal de réquisition auprès de la compagnie aérienne Emirates sur les déplacements d'AVB depuis le 01/01/2022 : relève 5 réservations effectuées et honorées, réglées par carte bancaire à l'exception d'un dossier du 19/09/2022 acquitté en espèces ; utilisation par AVB de titres de voyage / nationalités de la Grenade, de Bulgarie et des Émirats arabes unis, adresse courriel de contact xprivate@ukr.net.</t>
+          <t>Procès-verbal de réquisition auprès de la compagnie aérienne Emirates sur les déplacements d'AVB depuis le 1er janvier 2022 : relève 5 réservations effectuées et honorées, réglées par carte bancaire à l'exception d'un dossier du 19 septembre 2022 acquitté en espèces ; utilisation par AVB de titres de voyage / nationalités de la Grenade, de Bulgarie et des Émirats arabes unis, adresse courriel de contact xprivate@ukr.net.</t>
         </is>
       </c>
     </row>
@@ -7280,7 +7280,7 @@
       </c>
       <c r="F240" s="3" t="inlineStr">
         <is>
-          <t>Contrat n° 1-2014/10 du 28/10/2014 liant Duncan Promotions Ltd à Fraser Corporation portant sur des prestations de marketing, correspondances associées et ordre de virement signé par AVB disposant du transfert de 15 000 EUR.</t>
+          <t>Contrat n° 1-2014/10 du 28 octobre 2014 liant Duncan Promotions Ltd à Fraser Corporation portant sur des prestations de marketing, correspondances associées et ordre de virement signé par AVB disposant du transfert de 15 000 EUR.</t>
         </is>
       </c>
     </row>
@@ -7312,7 +7312,7 @@
       </c>
       <c r="F241" s="3" t="inlineStr">
         <is>
-          <t>Procès-verbal de réception, remis par les enquêteurs ukrainiens dans le cadre de l'ÉCI, de la copie de la demande d'entraide judiciaire (CRI) transmise le 13/06/2024 par l'Ukraine aux autorités de Monaco.</t>
+          <t>Procès-verbal de réception, remis par les enquêteurs ukrainiens dans le cadre de l'ÉCI, de la copie de la demande d'entraide judiciaire (CRI) transmise le 13 juin 2024 par l'Ukraine aux autorités de Monaco.</t>
         </is>
       </c>
     </row>
@@ -7344,7 +7344,7 @@
       </c>
       <c r="F242" s="3" t="inlineStr">
         <is>
-          <t>Procès-verbal d'analyse des informations figurant dans la demande d'entraide judiciaire ukrainienne du 19/04/2024 adressée à Monaco. L'enquête consigne la thèse ukrainienne relative à la sous-évaluation d'actifs de MS lors de la privatisation, à la procédure pénale disjointe visant M. Pryadko, ainsi qu'aux épisodes d'exportation de composants et moteurs de MS vers la Fédération de Russie via la Chine avec la participation de VAB et de M. Dziouba.</t>
+          <t>Procès-verbal d'analyse des informations figurant dans la demande d'entraide judiciaire ukrainienne du 19 avril 2024 adressée à Monaco. L'enquête consigne la thèse ukrainienne relative à la sous-évaluation d'actifs de MS lors de la privatisation, à la procédure pénale disjointe visant M. Pryadko, ainsi qu'aux épisodes d'exportation de composants et moteurs de MS vers la Fédération de Russie via la Chine avec la participation de VAB et de M. Dziouba.</t>
         </is>
       </c>
     </row>
@@ -7376,7 +7376,7 @@
       </c>
       <c r="F243" s="3" t="inlineStr">
         <is>
-          <t>Procès-verbal d'examen de la transmission de données fiscales ukrainiennes en date du 26/06/2024. Les enquêteurs relèvent que la structure des fichiers est strictement identique aux éléments précédemment communiqués et analysés le 28/06/2024.</t>
+          <t>Procès-verbal d'examen de la transmission de données fiscales ukrainiennes en date du 26 juin 2024. Les enquêteurs relèvent que la structure des fichiers est strictement identique aux éléments précédemment communiqués et analysés le 28 juin 2024.</t>
         </is>
       </c>
     </row>
@@ -7596,7 +7596,7 @@
       </c>
       <c r="F250" s="3" t="inlineStr">
         <is>
-          <t>Procès-verbal de recoupement bancaire afférent au virement de 293 239,27 EUR exécuté le 12/04/2016. Constate qu'AVB a remis au gestionnaire de son compte monégasque deux justificatifs : un extrait de l'acte notarié d'acquisition d'un appartement, d'un garage et d'un stationnement deux-roues dans une résidence sise à Nice.</t>
+          <t>Procès-verbal de recoupement bancaire afférent au virement de 293 239,27 EUR exécuté le 12 avril 2016. Constate qu'AVB a remis au gestionnaire de son compte monégasque deux justificatifs : un extrait de l'acte notarié d'acquisition d'un appartement, d'un garage et d'un stationnement deux-roues dans une résidence sise à Nice.</t>
         </is>
       </c>
     </row>
@@ -7880,7 +7880,7 @@
       </c>
       <c r="F259" s="7" t="inlineStr">
         <is>
-          <t>Procès-verbal d'audition de témoin d'Alain René Vergne, agent immobilier et proche d'AVB (Anton Vyacheslavovych Boguslayev). M. Vergne déclare connaître AVB depuis 2017 environ, s'être initialement occupé de la gestion de ses véhicules automobiles à Monaco, avoir entretenu des liens personnels avec lui, avoir participé à la surveillance matérielle du Domaine de Cuiros, avoir perçu d'AVB la somme de 3 500 EUR par mois en espèces jusqu'en 2024, avoir logé gratuitement dans une maison située sur la propriété de Cuiros, et avoir eu connaissance d'une partie du patrimoine d'AVB à Monaco et en France, tout en réfutant toute intervention dans la majorité des transactions d'acquisition.</t>
+          <t>Procès-verbal d'audition de témoin d'Alain René Vergne, agent immobilier et proche d'AVB (Oleksandr Vyacheslavovych Boguslayev). M. Vergne déclare connaître AVB depuis 2017 environ, s'être initialement occupé de la gestion de ses véhicules automobiles à Monaco, avoir entretenu des liens personnels avec lui, avoir participé à la surveillance matérielle du Domaine de Cuiros, avoir perçu d'AVB la somme de 3 500 EUR par mois en espèces jusqu'en 2024, avoir logé gratuitement dans une maison située sur la propriété de Cuiros, et avoir eu connaissance d'une partie du patrimoine d'AVB à Monaco et en France, tout en réfutant toute intervention dans la majorité des transactions d'acquisition.</t>
         </is>
       </c>
     </row>
@@ -8424,7 +8424,7 @@
       </c>
       <c r="F276" s="7" t="inlineStr">
         <is>
-          <t>Procès-verbal de versement et de traduction automatisée d'un article ukrainien du 23/04/2025 issu du média « Sudovyi Reporter ». L'article expose des fournitures de matériels de MS au complexe militaro-industriel de la Fédération de Russie postérieures au décret d'embargo, le recours à des sociétés intermédiaires en Chine et aux Émirats arabes unis, l'importation de pièces en Russie et la qualification pénale retenue au titre du Code pénal d'Ukraine (CP).</t>
+          <t>Procès-verbal de versement et de traduction automatisée d'un article ukrainien du 23 avril 2025 issu du média « Sudovyi Reporter ». L'article expose des fournitures de matériels de MS au complexe militaro-industriel de la Fédération de Russie postérieures au décret d'embargo, le recours à des sociétés intermédiaires en Chine et aux Émirats arabes unis, l'importation de pièces en Russie et la qualification pénale retenue au titre du Code pénal d'Ukraine (CP).</t>
         </is>
       </c>
     </row>
@@ -8483,12 +8483,12 @@
       </c>
       <c r="E278" s="7" t="inlineStr">
         <is>
-          <t>AVB ; convention d'entiercement ; 21/12/2015 ; UBI Banca ; Skyrizon ; Reckoner ; Argio ; Laterson ; Katran ; Stamio ; Taladin ; Calloway ; Longwizard ; Enfields ; Granum ; Waldo</t>
+          <t>AVB ; convention d'entiercement ; 21 décembre 2015 ; UBI Banca ; Skyrizon ; Reckoner ; Argio ; Laterson ; Katran ; Stamio ; Taladin ; Calloway ; Longwizard ; Enfields ; Granum ; Waldo</t>
         </is>
       </c>
       <c r="F278" s="7" t="inlineStr">
         <is>
-          <t>Procès-verbal d'examen de 9 originaux de la convention d'entiercement (Escrow Agreement) du 21/12/2015 : acheteurs — Skyrizon, Reckoner et Argio ; vendeurs — Laterson, Katran, Stamio, Taladin, Calloway et Longwizard ; agent d'entiercement — UBI Banca International. AVB est désigné comme mandataire des six sociétés cédantes ; les enquêteurs constatent que l'ensemble des 9 originaux de l'accord ont été découverts en sa possession.</t>
+          <t>Procès-verbal d'examen de 9 originaux de la convention d'entiercement (Escrow Agreement) du 21 décembre 2015 : acheteurs — Skyrizon, Reckoner et Argio ; vendeurs — Laterson, Katran, Stamio, Taladin, Calloway et Longwizard ; agent d'entiercement — UBI Banca International. AVB est désigné comme mandataire des six sociétés cédantes ; les enquêteurs constatent que l'ensemble des 9 originaux de l'accord ont été découverts en sa possession.</t>
         </is>
       </c>
     </row>
@@ -8579,12 +8579,12 @@
       </c>
       <c r="E281" s="7" t="inlineStr">
         <is>
-          <t>Convention d'entiercement ; 21/12/2015 ; VAB ; Likraton Enterprises ; UBI Banca Luxembourg ; compte d'entiercement</t>
+          <t>Convention d'entiercement ; 21 décembre 2015 ; VAB ; Likraton Enterprises ; UBI Banca Luxembourg ; compte d'entiercement</t>
         </is>
       </c>
       <c r="F281" s="7" t="inlineStr">
         <is>
-          <t>Procès-verbal d'examen de deux exemplaires de la convention d'entiercement du 21/12/2015 relative au Project Zoom II : VAB (Vyacheslav Oleksandrovych Boguslayev) — cédant, Likraton Enterprises Limited — acquéreur, UBI Banca Luxembourg — agent d'entiercement ; prévoyant l'ouverture de comptes séquestres libellés en EUR et en USD.</t>
+          <t>Procès-verbal d'examen de deux exemplaires de la convention d'entiercement du 21 décembre 2015 relative au Project Zoom II : VAB (Vyacheslav Oleksandrovych Boguslayev) — cédant, Likraton Enterprises Limited — acquéreur, UBI Banca Luxembourg — agent d'entiercement ; prévoyant l'ouverture de comptes séquestres libellés en EUR et en USD.</t>
         </is>
       </c>
     </row>
@@ -8611,12 +8611,12 @@
       </c>
       <c r="E282" s="7" t="inlineStr">
         <is>
-          <t>Convention d'entiercement ; 21/12/2015 ; 582 000 000 USD ; 100 000 000 USD ; UBI Banca ; Skyrizon ; Reckoner ; Argio ; Laterson ; Katran ; Stamio ; Taladin ; Calloway ; Longwizard ; MS</t>
+          <t>Convention d'entiercement ; 21 décembre 2015 ; 582 000 000 USD ; 100 000 000 USD ; UBI Banca ; Skyrizon ; Reckoner ; Argio ; Laterson ; Katran ; Stamio ; Taladin ; Calloway ; Longwizard ; MS</t>
         </is>
       </c>
       <c r="F282" s="7" t="inlineStr">
         <is>
-          <t>Procès-verbal d'examen de neuf exemplaires de la convention d'entiercement du 21/12/2015 relative à la cession d'actions de MS : séquestre portant sur 582 000 000 USD, conditions de répartition des fonds entre les vendeurs et modalités de libération ; la convention prévoit également un prêt d'investissement consenti à MS pour un montant de 100 000 000 USD sur 10 ans au taux de 0,3 %.</t>
+          <t>Procès-verbal d'examen de neuf exemplaires de la convention d'entiercement du 21 décembre 2015 relative à la cession d'actions de MS : séquestre portant sur 582 000 000 USD, conditions de répartition des fonds entre les vendeurs et modalités de libération ; la convention prévoit également un prêt d'investissement consenti à MS pour un montant de 100 000 000 USD sur 10 ans au taux de 0,3 %.</t>
         </is>
       </c>
     </row>
@@ -8643,12 +8643,12 @@
       </c>
       <c r="E283" s="7" t="inlineStr">
         <is>
-          <t>Letter of Undertaking ; 65 % ; 582 000 000 USD ; 43 000 000 USD ; 107 000 000 USD ; 21/12/2015 ; VAB ; Laterson ; Katran ; Stamio ; Taladin ; Calloway ; Longwizard ; Skyrizon ; Reckoner ; Argio ; Likraton</t>
+          <t>Letter of Undertaking ; 65 % ; 582 000 000 USD ; 43 000 000 USD ; 107 000 000 USD ; 21 décembre 2015 ; VAB ; Laterson ; Katran ; Stamio ; Taladin ; Calloway ; Longwizard ; Skyrizon ; Reckoner ; Argio ; Likraton</t>
         </is>
       </c>
       <c r="F283" s="7" t="inlineStr">
         <is>
-          <t>Procès-verbal d'examen de sept originaux de la lettre d'engagement (Letter of Undertaking) du 21/12/2015 portant sur la vente de 65 % des actions du groupe MS : désignation des cédants et des acquéreurs, prix total fixé à 582 000 000 USD, premier acompte de 43 000 000 USD et engagement des vendeurs de reverser aux acheteurs la somme de 107 000 000 USD consécutivement au versement du prêt d'investissement.</t>
+          <t>Procès-verbal d'examen de sept originaux de la lettre d'engagement (Letter of Undertaking) du 21 décembre 2015 portant sur la vente de 65 % des actions du groupe MS : désignation des cédants et des acquéreurs, prix total fixé à 582 000 000 USD, premier acompte de 43 000 000 USD et engagement des vendeurs de reverser aux acheteurs la somme de 107 000 000 USD consécutivement au versement du prêt d'investissement.</t>
         </is>
       </c>
     </row>
@@ -8675,12 +8675,12 @@
       </c>
       <c r="E284" s="7" t="inlineStr">
         <is>
-          <t>Accord-cadre ; 21/12/2015 ; Laterson ; Katran ; Stamio ; Taladin ; Calloway ; Longwizard ; Skyrizon ; Reckoner ; Argio ; structure MS ; ME ; Geoford ; 100 000 000 USD</t>
+          <t>Accord-cadre ; 21 décembre 2015 ; Laterson ; Katran ; Stamio ; Taladin ; Calloway ; Longwizard ; Skyrizon ; Reckoner ; Argio ; structure MS ; ME ; Geoford ; 100 000 000 USD</t>
         </is>
       </c>
       <c r="F284" s="7" t="inlineStr">
         <is>
-          <t>Procès-verbal d'examen de l'accord-cadre du 29/05/2015 dans sa version modifiée du 21/12/2015 : répartition des participations au capital de MS et du prix entre les cédants et cessionnaires, inventaire des entités du groupe MS et de leur schéma de détention (incluant ME) ; conditions d'octroi du prêt d'investissement de 100 000 000 USD consenti à MS et affectation de ces fonds.</t>
+          <t>Procès-verbal d'examen de l'accord-cadre du 29 mai 2015 dans sa version modifiée du 21 décembre 2015 : répartition des participations au capital de MS et du prix entre les cédants et cessionnaires, inventaire des entités du groupe MS et de leur schéma de détention (incluant ME) ; conditions d'octroi du prêt d'investissement de 100 000 000 USD consenti à MS et affectation de ces fonds.</t>
         </is>
       </c>
     </row>
@@ -8712,7 +8712,7 @@
       </c>
       <c r="F285" s="7" t="inlineStr">
         <is>
-          <t>Procès-verbal d'examen des documents saisis dans le coffre-fort d'UBP Monaco : pièces relatives à Geoford LLP, Tabernus Corp, Aldon Business Inc., Dunkan Promotions Ltd., MS et aux comptes bancaires ; actes de cession d'actions de MS en date du 07/07/2016, dont 9,99 % au profit de Likraton Enterprises pour 28 638 000 USD. Les enquêteurs mettent en regard les relevés bancaires de Motor Bank portant sur 14 362 000 USD et 28 638 000 USD (soit 43 000 000 USD au total) avec les deux actes de transfert de titres.</t>
+          <t>Procès-verbal d'examen des documents saisis dans le coffre-fort d'UBP Monaco : pièces relatives à Geoford LLP, Tabernus Corp, Aldon Business Inc., Dunkan Promotions Ltd., MS et aux comptes bancaires ; actes de cession d'actions de MS en date du 7 juillet 2016, dont 9,99 % au profit de Likraton Enterprises pour 28 638 000 USD. Les enquêteurs mettent en regard les relevés bancaires de Motor Bank portant sur 14 362 000 USD et 28 638 000 USD (soit 43 000 000 USD au total) avec les deux actes de transfert de titres.</t>
         </is>
       </c>
     </row>
@@ -8803,12 +8803,12 @@
       </c>
       <c r="E288" s="7" t="inlineStr">
         <is>
-          <t>AVB ; Katsylo ; A vendre.docx ; 05/05/2014 ; schéma de transaction ; 49,8 % ; 2 % ; 15 % ; entiercement ; due diligence ; AMKU</t>
+          <t>AVB ; Katsylo ; A vendre.docx ; 5 mai 2014 ; schéma de transaction ; 49,8 % ; 2 % ; 15 % ; entiercement ; due diligence ; AMKU</t>
         </is>
       </c>
       <c r="F288" s="7" t="inlineStr">
         <is>
-          <t>Procès-verbal d'examen d'un message électronique de M. Katsylo adressé à AVB le 05/05/2014 et du fichier joint « A vendre.docx » détaillant un montage transactionnel en trois temps : cession initiale de 49,8 % des actions, rachat en bourse de 2 % par l'acheteur, puis acquisition subséquente du solde des titres. Le document détaille l'entiercement, la due diligence et les contrats de cession ; il précise que l'autorisation de concentration de l'AMKU (Comité anti-monopole d'Ukraine) constitue une condition du règlement final tout en envisageant de clôturer la cession avant toute notification formelle à l'AMKU.</t>
+          <t>Procès-verbal d'examen d'un message électronique de M. Katsylo adressé à AVB le 5 mai 2014 et du fichier joint « A vendre.docx » détaillant un montage transactionnel en trois temps : cession initiale de 49,8 % des actions, rachat en bourse de 2 % par l'acheteur, puis acquisition subséquente du solde des titres. Le document détaille l'entiercement, la due diligence et les contrats de cession ; il précise que l'autorisation de concentration de l'AMKU (Comité anti-monopole d'Ukraine) constitue une condition du règlement final tout en envisageant de clôturer la cession avant toute notification formelle à l'AMKU.</t>
         </is>
       </c>
     </row>
@@ -8931,12 +8931,12 @@
       </c>
       <c r="E292" s="7" t="inlineStr">
         <is>
-          <t>Project Zoom ; courriel ; 14/11/2014 ; ordinateur</t>
+          <t>Project Zoom ; courriel ; 14 novembre 2014 ; ordinateur</t>
         </is>
       </c>
       <c r="F292" s="8" t="inlineStr">
         <is>
-          <t>Procès-verbal d'exploitation de données informatiques : message électronique du 14/11/2014 relatif au Project Zoom.</t>
+          <t>Procès-verbal d'exploitation de données informatiques : message électronique du 14 novembre 2014 relatif au Project Zoom.</t>
         </is>
       </c>
     </row>
@@ -8963,12 +8963,12 @@
       </c>
       <c r="E293" s="7" t="inlineStr">
         <is>
-          <t>Project Zoom ; courriel ; 29/12/2015 ; 50 % ; ordinateur</t>
+          <t>Project Zoom ; courriel ; 29 décembre 2015 ; 50 % ; ordinateur</t>
         </is>
       </c>
       <c r="F293" s="7" t="inlineStr">
         <is>
-          <t>Procès-verbal d'exploitation de données informatiques : message électronique du 29/12/2015 relatif au Project Zoom comportant la mention 50 %.</t>
+          <t>Procès-verbal d'exploitation de données informatiques : message électronique du 29 décembre 2015 relatif au Project Zoom comportant la mention 50 %.</t>
         </is>
       </c>
     </row>
@@ -8995,12 +8995,12 @@
       </c>
       <c r="E294" s="7" t="inlineStr">
         <is>
-          <t>Project Zoom ; courriel ; 29/12/2015 ; 15 % ; ordinateur</t>
+          <t>Project Zoom ; courriel ; 29 décembre 2015 ; 15 % ; ordinateur</t>
         </is>
       </c>
       <c r="F294" s="7" t="inlineStr">
         <is>
-          <t>Procès-verbal d'exploitation de données informatiques : message électronique du 29/12/2015 relatif au Project Zoom comportant la mention 15 %.</t>
+          <t>Procès-verbal d'exploitation de données informatiques : message électronique du 29 décembre 2015 relatif au Project Zoom comportant la mention 15 %.</t>
         </is>
       </c>
     </row>
@@ -9027,12 +9027,12 @@
       </c>
       <c r="E295" s="7" t="inlineStr">
         <is>
-          <t>AVB ; Katsylo ; Chine ; usine ; 16/12/2015 ; 28/12/2015 ; transfert de fonds</t>
+          <t>AVB ; Katsylo ; Chine ; usine ; 16 décembre 2015 ; 28 décembre 2015 ; transfert de fonds</t>
         </is>
       </c>
       <c r="F295" s="7" t="inlineStr">
         <is>
-          <t>Procès-verbal d'examen des échanges entre M. Katsylo et AVB en date du 16/12/2015 : invitation officielle adressée à AVB à l'occasion de la cérémonie de pose de la première pierre de l'usine en Chine le 28/12/2015 ; AVB indique en retour qu'il répondra favorablement à cette invitation dès la réalisation effective du transfert de fonds.</t>
+          <t>Procès-verbal d'examen des échanges entre M. Katsylo et AVB en date du 16 décembre 2015 : invitation officielle adressée à AVB à l'occasion de la cérémonie de pose de la première pierre de l'usine en Chine le 28 décembre 2015 ; AVB indique en retour qu'il répondra favorablement à cette invitation dès la réalisation effective du transfert de fonds.</t>
         </is>
       </c>
     </row>
@@ -9059,12 +9059,12 @@
       </c>
       <c r="E296" s="7" t="inlineStr">
         <is>
-          <t>AVB ; Katsylo ; Ilya Muchnyk ; DLA Piper ; protocole d'accord 17/05/2014 ; avenant ; Laterson ; Skyrizon ; Enfields ; Granum ; Waldo ; HSBC ; entiercement ; KYC ; due diligence ; 25 000 000 USD ; 16 000 000 USD ; 9 000 000 USD ; Chine</t>
+          <t>AVB ; Katsylo ; Ilya Muchnyk ; DLA Piper ; protocole d'accord 17 mai 2014 ; avenant ; Laterson ; Skyrizon ; Enfields ; Granum ; Waldo ; HSBC ; entiercement ; KYC ; due diligence ; 25 000 000 USD ; 16 000 000 USD ; 9 000 000 USD ; Chine</t>
         </is>
       </c>
       <c r="F296" s="7" t="inlineStr">
         <is>
-          <t>Procès-verbal d'examen de la correspondance de juin–juillet 2014 entre M. Katsylo, AVB et les représentants du cabinet DLA Piper relative au Project Zoom : modifications apportées au protocole d'accord (MOU) du 17/05/2014, organisation de l'entiercement via HSBC, diligences KYC et due diligence, obtention de l'agrément des autorités réglementaires chinoises pour la conversion de devises, et ventilation du règlement de 25 000 000 USD en deux tranches de 16 000 000 USD et 9 000 000 USD. Les enquêteurs rattachent ces échanges à la première phase du Project Zoom, à savoir la cession de Laterson au profit de Skyrizon.</t>
+          <t>Procès-verbal d'examen de la correspondance de juin–juillet 2014 entre M. Katsylo, AVB et les représentants du cabinet DLA Piper relative au Project Zoom : modifications apportées au protocole d'accord (MOU) du 17 mai 2014, organisation de l'entiercement via HSBC, diligences KYC et due diligence, obtention de l'agrément des autorités réglementaires chinoises pour la conversion de devises, et ventilation du règlement de 25 000 000 USD en deux tranches de 16 000 000 USD et 9 000 000 USD. Les enquêteurs rattachent ces échanges à la première phase du Project Zoom, à savoir la cession de Laterson au profit de Skyrizon.</t>
         </is>
       </c>
     </row>
@@ -9091,12 +9091,12 @@
       </c>
       <c r="E297" s="7" t="inlineStr">
         <is>
-          <t>AVB ; Katsylo ; Laterson ; Skyrizon ; UBI Banca ; UBO ; compte d'entiercement ; Roberto Rampino ; 05/11/2014</t>
+          <t>AVB ; Katsylo ; Laterson ; Skyrizon ; UBI Banca ; UBO ; compte d'entiercement ; Roberto Rampino ; 5 novembre 2014</t>
         </is>
       </c>
       <c r="F297" s="7" t="inlineStr">
         <is>
-          <t>Procès-verbal d'examen d'un message d'UBI Banca du 05/11/2014 ayant pour objet « Compte d'entiercement Laterson / Skyrizon », adressé à M. Katsylo et à AVB : l'établissement bancaire sollicite une référence bancaire concernant le bénéficiaire effectif (UBO) de Laterson. L'autorité d'enquête souligne que la notification directe de cette demande à AVB et à son conseil constitue un indice fort de son contrôle effectif sur la société Laterson.</t>
+          <t>Procès-verbal d'examen du courrier d'UBI Banca du 5 novembre 2014 ayant pour objet « Compte séquestre Laterson / Skyrizon », adressé à Katsylo et à AVB : la banque sollicite une recommandation bancaire concernant l'UBO de Laterson. L'enquête indique séparément que l'envoi de cette demande directement à AVB et à son avocat témoigne, selon les enquêteurs, d'un lien entre AVB et Laterson.</t>
         </is>
       </c>
     </row>
@@ -9123,12 +9123,12 @@
       </c>
       <c r="E298" s="7" t="inlineStr">
         <is>
-          <t>AVB ; Katsylo ; Ilya Muchnyk ; DLA Piper ; Wang Jing ; Skyrizon ; protocole d'accord 17/05/2014 ; avenant 19/12/2014 ; 65 % ; 15 % ; entiercement ; 25 000 000 USD ; AMKU</t>
+          <t>AVB ; Katsylo ; Ilya Muchnyk ; DLA Piper ; Wang Jing ; Skyrizon ; protocole d'accord 17 mai 2014 ; avenant 19 décembre 2014 ; 65 % ; 15 % ; entiercement ; 25 000 000 USD ; AMKU</t>
         </is>
       </c>
       <c r="F298" s="7" t="inlineStr">
         <is>
-          <t>Procès-verbal d'examen d'un courriel du 20/12/2014 et de l'avenant (Amendment Agreement) du 19/12/2014 signé par Wang Jing, modifiant le protocole d'accord du 17/05/2014. L'acte prévoit une transaction avec des cédants détenant plus de 65 % de MS, un paiement séquestré de 25 000 000 USD et l'acquisition ultérieure d'un bloc supplémentaire de 15 % d'actions ; il stipule expressément que cette seconde acquisition ne requiert aucune autorisation de concentration délivrée par l'AMKU (Comité anti-monopole d'Ukraine).</t>
+          <t>Procès-verbal d'examen d'un courriel du 20 décembre 2014 et de l'avenant (Amendment Agreement) du 19 décembre 2014 signé par Wang Jing, modifiant le protocole d'accord du 17 mai 2014. L'acte prévoit une transaction avec des cédants détenant plus de 65 % de MS, un paiement séquestré de 25 000 000 USD et l'acquisition ultérieure d'un bloc supplémentaire de 15 % d'actions ; il stipule expressément que cette seconde acquisition ne requiert aucune autorisation de concentration délivrée par l'AMKU (Comité anti-monopole d'Ukraine).</t>
         </is>
       </c>
     </row>
@@ -9155,12 +9155,12 @@
       </c>
       <c r="E299" s="7" t="inlineStr">
         <is>
-          <t>AVB ; Katsylo ; accord-cadre ; 01/04/2015 ; entiercement ; restructuration ; due diligence ; contrat de gestion ; garanties ; 15 % ; structure de la transaction</t>
+          <t>AVB ; Katsylo ; accord-cadre ; 1er avril 2015 ; entiercement ; restructuration ; due diligence ; contrat de gestion ; garanties ; 15 % ; structure de la transaction</t>
         </is>
       </c>
       <c r="F299" s="7" t="inlineStr">
         <is>
-          <t>Procès-verbal d'examen d'une correspondance de M. Katsylo adressée à AVB le 01/04/2015 analysant le projet reçu d'accord-cadre : exposé de la structure contractuelle proposée par les acheteurs et contre-propositions relatives à la réorganisation des entités, à l'entiercement, à la due diligence, à la convention de gestion, aux garanties, aux modalités de closing et à la cession distincte d'un bloc de 15 % du capital.</t>
+          <t>Procès-verbal d'examen d'une correspondance de M. Katsylo adressée à AVB le 1er avril 2015 analysant le projet reçu d'accord-cadre : exposé de la structure contractuelle proposée par les acheteurs et contre-propositions relatives à la réorganisation des entités, à l'entiercement, à la due diligence, à la convention de gestion, aux garanties, aux modalités de closing et à la cession distincte d'un bloc de 15 % du capital.</t>
         </is>
       </c>
     </row>
@@ -9187,12 +9187,12 @@
       </c>
       <c r="E300" s="7" t="inlineStr">
         <is>
-          <t>UBI ; entiercement ; 28/04/2015 ; déblocage des fonds ; ordinateur</t>
+          <t>UBI ; entiercement ; 28 avril 2015 ; déblocage des fonds ; ordinateur</t>
         </is>
       </c>
       <c r="F300" s="7" t="inlineStr">
         <is>
-          <t>Procès-verbal d'exploitation de données informatiques : message du 28/04/2015 attestant de la confirmation par UBI de la libération des fonds placés sous séquestre / entiercement.</t>
+          <t>Procès-verbal d'exploitation de données informatiques : message du 28 avril 2015 attestant de la confirmation par UBI de la libération des fonds placés sous séquestre / entiercement.</t>
         </is>
       </c>
     </row>
@@ -9256,7 +9256,7 @@
       </c>
       <c r="F302" s="7" t="inlineStr">
         <is>
-          <t>Procès-verbal d'exploitation du matériel informatique utilisé selon l'enquête par AVB : identification de ses adresses électroniques et de documents personnels. Parmi ceux-ci figurent une attestation de ME en date du 09/07/2016 mentionnant ses fonctions de directeur depuis 2008, un certificat de résidence fiscale aux Émirats arabes unis, ainsi que des pièces afférentes à l'obtention de la nationalité et de la résidence permanente à la Grenade.</t>
+          <t>Procès-verbal d'exploitation du matériel informatique utilisé selon l'enquête par AVB : identification de ses adresses électroniques et de documents personnels. Parmi ceux-ci figurent une attestation de ME en date du 9 juillet 2016 mentionnant ses fonctions de directeur depuis 2008, un certificat de résidence fiscale aux Émirats arabes unis, ainsi que des pièces afférentes à l'obtention de la nationalité et de la résidence permanente à la Grenade.</t>
         </is>
       </c>
     </row>
@@ -9608,7 +9608,7 @@
       </c>
       <c r="F313" s="7" t="inlineStr">
         <is>
-          <t>Bordereaux de transmission et actes de remise de documents entre Astapov &amp; Partners et DLA Piper Ukraine : statuts, actes de constitution, registres sociaux et sceaux de Croftdale, Montagne, Waldo, Enfields, BH Helena et Granum, ainsi que contrats de services et pièces relatives au « Project Zoom », incluant la date de clôture (Completion Date) et les actes de renonciation (Waiver) du 27/01/2016 afférents à Laterson, Katran, Stamio, Taladin, Calloway et Longwizard.</t>
+          <t>Bordereaux de transmission et actes de remise de documents entre Astapov &amp; Partners et DLA Piper Ukraine : statuts, actes de constitution, registres sociaux et sceaux de Croftdale, Montagne, Waldo, Enfields, BH Helena et Granum, ainsi que contrats de services et pièces relatives au « Project Zoom », incluant la date de clôture (Completion Date) et les actes de renonciation (Waiver) du 27 janvier 2016 afférents à Laterson, Katran, Stamio, Taladin, Calloway et Longwizard.</t>
         </is>
       </c>
     </row>
@@ -9800,7 +9800,7 @@
       </c>
       <c r="F319" s="7" t="inlineStr">
         <is>
-          <t>Procès-verbal de versement de traductions certifiées d'actes de procédure ukrainiens : ordonnance du tribunal de district Shevchenkivsky de Kyiv en date du 09/05/2024 autorisant l'accès temporaire aux données fiscales de VAB, d'AVB et de M. Kononenko auprès du Service national des impôts d'Ukraine (DPS) ; pièces d'exécution afférentes ; procès-verbal d'accès temporaire du 29/05/2024 avec inventaire des pièces remises. Les motifs de la requête font expressément état des données de la procédure pénale française et des commissions rogatoires internationales.</t>
+          <t>Procès-verbal de versement de traductions certifiées d'actes de procédure ukrainiens : ordonnance du tribunal de district Shevchenkivsky de Kyiv en date du 9 mai 2024 autorisant l'accès temporaire aux données fiscales de VAB, d'AVB et de M. Kononenko auprès du Service national des impôts d'Ukraine (DPS) ; pièces d'exécution afférentes ; procès-verbal d'accès temporaire du 29 mai 2024 avec inventaire des pièces remises. Les motifs de la requête font expressément état des données de la procédure pénale française et des commissions rogatoires internationales.</t>
         </is>
       </c>
     </row>
@@ -9987,12 +9987,12 @@
       </c>
       <c r="E325" s="7" t="inlineStr">
         <is>
-          <t>Avenant ; protocole d'accord (MOU) ; 17/05/2014 ; traduction</t>
+          <t>Avenant ; protocole d'accord (MOU) ; 17 mai 2014 ; traduction</t>
         </is>
       </c>
       <c r="F325" s="7" t="inlineStr">
         <is>
-          <t>Procès-verbal d'examen du projet d'avenant (Amendment Agreement) au protocole d'accord du 17/05/2014, adressé par M. Katsylo à AVB le 27/06/2014 après transmission par DLA Piper. L'acte concerne les cédants détenant plus de 65 % des actions de MS ainsi que Skyrizon / Wang Jing en qualité d'acquéreur, et redéfinit l'échéancier des règlements. Les enquêteurs relèvent que cet exemplaire n'a pas été signé par les parties.</t>
+          <t>Procès-verbal d'examen du projet d'avenant (Amendment Agreement) au protocole d'accord du 17 mai 2014, adressé par M. Katsylo à AVB le 27 juin 2014 après transmission par DLA Piper. L'acte concerne les cédants détenant plus de 65 % des actions de MS ainsi que Skyrizon / Wang Jing en qualité d'acquéreur, et redéfinit l'échéancier des règlements. Les enquêteurs relèvent que cet exemplaire n'a pas été signé par les parties.</t>
         </is>
       </c>
     </row>
@@ -10019,12 +10019,12 @@
       </c>
       <c r="E326" s="7" t="inlineStr">
         <is>
-          <t>AVB ; Wang Jing ; Katsylo ; Skyrizon ; UBI Banca ; 25 000 000 USD ; 250 000 000 USD ; Chine ; protocole d'accord (MOU) ; 20/12/2014 ; Project Zoom</t>
+          <t>AVB ; Wang Jing ; Katsylo ; Skyrizon ; UBI Banca ; 25 000 000 USD ; 250 000 000 USD ; Chine ; protocole d'accord (MOU) ; 20 décembre 2014 ; Project Zoom</t>
         </is>
       </c>
       <c r="F326" s="7" t="inlineStr">
         <is>
-          <t>Procès-verbal d'examen de la lettre de Wang Jing en date du 11/01/2015 adressée à AVB : l'auteur rappelle la signature le 20/12/2014 des avenants au protocole d'accord, l'ouverture de compte auprès d'UBI Banca et le premier versement de 25 000 000 USD intervenu le 29/12/2014 ; il sollicite le développement de la coopération industrielle et propose un plan d'investissement d'environ 250 000 000 USD sur trois ans dans la recherche et développement et l'appareil productif et commercial de MS en Chine.</t>
+          <t>Procès-verbal d'examen de la lettre de Wang Jing en date du 11 janvier 2015 adressée à AVB : l'auteur rappelle la signature le 20 décembre 2014 des avenants au protocole d'accord, l'ouverture de compte auprès d'UBI Banca et le premier versement de 25 000 000 USD intervenu le 29 décembre 2014 ; il sollicite le développement de la coopération industrielle et propose un plan d'investissement d'environ 250 000 000 USD sur trois ans dans la recherche et développement et l'appareil productif et commercial de MS en Chine.</t>
         </is>
       </c>
     </row>
@@ -10083,12 +10083,12 @@
       </c>
       <c r="E328" s="7" t="inlineStr">
         <is>
-          <t>AVB ; Wang Jing ; Skyrizon ; protocole d'accord 17/05/2014 ; avenant ; 19/12/2014 ; AMKU ; concentration</t>
+          <t>AVB ; Wang Jing ; Skyrizon ; protocole d'accord 17 mai 2014 ; avenant ; 19 décembre 2014 ; AMKU ; concentration</t>
         </is>
       </c>
       <c r="F328" s="7" t="inlineStr">
         <is>
-          <t>Procès-verbal d'examen de l'Amendment Agreement du 19/12/2014 au MOU du 17/05/2014 signé par Wang Jing. Le document contient explicitement une disposition selon laquelle les parties confirment qu'une autorisation de concentration de l'AMKU (Comité anti-monopole d'Ukraine) n'est pas nécessaire pour l'acquisition d'actions concernée. L'enquête considère cette disposition comme soulevant une question quant au respect des exigences anti-monopole.</t>
+          <t>Procès-verbal d'examen de l'Amendment Agreement du 19 décembre 2014 au MOU du 17 mai 2014 signé par Wang Jing. Le document contient explicitement une disposition selon laquelle les parties confirment qu'une autorisation de concentration de l'AMKU (Comité anti-monopole d'Ukraine) n'est pas nécessaire pour l'acquisition d'actions concernée. L'enquête considère cette disposition comme soulevant une question quant au respect des exigences anti-monopole.</t>
         </is>
       </c>
     </row>
@@ -10147,12 +10147,12 @@
       </c>
       <c r="E330" s="7" t="inlineStr">
         <is>
-          <t>Evgeniy Vnukov ; AVB ; courriel ; 04/07/2016 ; traduction</t>
+          <t>Evgeniy Vnukov ; AVB ; courriel ; 4 juillet 2016 ; traduction</t>
         </is>
       </c>
       <c r="F330" s="7" t="inlineStr">
         <is>
-          <t>Procès-verbal d'examen de la traduction du russe de la correspondance par courriel échangée entre M. Vnukov et AVB en date du 04/07/2016.</t>
+          <t>Procès-verbal d'examen de la traduction du russe de la correspondance par courriel échangée entre M. Vnukov et AVB en date du 4 juillet 2016.</t>
         </is>
       </c>
     </row>
@@ -10179,12 +10179,12 @@
       </c>
       <c r="E331" s="7" t="inlineStr">
         <is>
-          <t>Nina Katsylo ; AVB ; courriel ; 01/04/2015 ; traduction</t>
+          <t>Nina Katsylo ; AVB ; courriel ; 1er avril 2015 ; traduction</t>
         </is>
       </c>
       <c r="F331" s="7" t="inlineStr">
         <is>
-          <t>Procès-verbal d'examen de la traduction du russe d'un courriel du 01/04/2015 entre Nina Katsylo et AVB.</t>
+          <t>Procès-verbal d'examen de la traduction du russe d'un courriel du 1er avril 2015 entre Nina Katsylo et AVB.</t>
         </is>
       </c>
     </row>
@@ -10243,12 +10243,12 @@
       </c>
       <c r="E333" s="7" t="inlineStr">
         <is>
-          <t>AVB ; Nina Katsylo ; AMKU ; Project Zoom ; courriel ; 05/05/2014 ; traduction</t>
+          <t>AVB ; Nina Katsylo ; AMKU ; Project Zoom ; courriel ; 5 mai 2014 ; traduction</t>
         </is>
       </c>
       <c r="F333" s="7" t="inlineStr">
         <is>
-          <t>Procès-verbal d'examen de la traduction du russe d'un courriel du 05/05/2014 entre AVB et Nina Katsylo portant sur les problématiques liées à l'AMKU (Comité anti-monopole d'Ukraine).</t>
+          <t>Procès-verbal d'examen de la traduction du russe d'un courriel du 5 mai 2014 entre AVB et Nina Katsylo portant sur les problématiques liées à l'AMKU (Comité anti-monopole d'Ukraine).</t>
         </is>
       </c>
     </row>
@@ -10275,12 +10275,12 @@
       </c>
       <c r="E334" s="7" t="inlineStr">
         <is>
-          <t>Nina Katsylo ; AVB ; Project Zoom ; risques ; courriel ; 24/02/2015 ; traduction</t>
+          <t>Nina Katsylo ; AVB ; Project Zoom ; risques ; courriel ; 24 février 2015 ; traduction</t>
         </is>
       </c>
       <c r="F334" s="7" t="inlineStr">
         <is>
-          <t>Procès-verbal d'examen de la correspondance du 24/02/2015 entre M. Katsylo et AVB sur les risques liés au « Project Zoom ». Est discutée la nécessité d'exclure Motor Bank du périmètre de la transaction, car son inclusion pourrait entraîner la publicité de la transaction, des conséquences politiques et juridiques ainsi qu'un risque de contestation/nullité de celle-ci. La question de l'acquisition des actions de MS sans autorisation préalable de l'AMKU est posée séparément et des options de sortie de Motor Bank avant ou après la clôture de la transaction sont proposées.</t>
+          <t>Procès-verbal d'examen de la correspondance du 24 février 2015 entre M. Katsylo et AVB sur les risques liés au « Project Zoom ». Est discutée la nécessité d'exclure Motor Bank du périmètre de la transaction, car son inclusion pourrait entraîner la publicité de la transaction, des conséquences politiques et juridiques ainsi qu'un risque de contestation/nullité de celle-ci. La question de l'acquisition des actions de MS sans autorisation préalable de l'AMKU est posée séparément et des options de sortie de Motor Bank avant ou après la clôture de la transaction sont proposées.</t>
         </is>
       </c>
     </row>
@@ -10307,12 +10307,12 @@
       </c>
       <c r="E335" s="7" t="inlineStr">
         <is>
-          <t>Nina Katsylo ; AVB ; Project Zoom ; gestion de fonds ; 01/05/2016 ; traduction</t>
+          <t>Nina Katsylo ; AVB ; Project Zoom ; gestion de fonds ; 1er mai 2016 ; traduction</t>
         </is>
       </c>
       <c r="F335" s="7" t="inlineStr">
         <is>
-          <t>Procès-verbal d'examen de la traduction du russe d'un courriel du 01/05/2016 entre Nina Katsylo et AVB traitant du placement et de la gestion des capitaux issus du Project Zoom.</t>
+          <t>Procès-verbal d'examen de la traduction du russe d'un courriel du 1er mai 2016 entre Nina Katsylo et AVB traitant du placement et de la gestion des capitaux issus du Project Zoom.</t>
         </is>
       </c>
     </row>
@@ -10339,12 +10339,12 @@
       </c>
       <c r="E336" s="7" t="inlineStr">
         <is>
-          <t>AVB ; Ukraine ; résidence fiscale ; mémorandum ; 31/05/2016 ; traduction</t>
+          <t>AVB ; Ukraine ; résidence fiscale ; mémorandum ; 31 mai 2016 ; traduction</t>
         </is>
       </c>
       <c r="F336" s="7" t="inlineStr">
         <is>
-          <t>Procès-verbal d'examen de la traduction du russe d'une consultation juridique du 31/05/2016 remise à AVB relative aux critères déterminant sa résidence fiscale en Ukraine.</t>
+          <t>Procès-verbal d'examen de la traduction du russe d'une consultation juridique du 31 mai 2016 remise à AVB relative aux critères déterminant sa résidence fiscale en Ukraine.</t>
         </is>
       </c>
     </row>
@@ -10408,7 +10408,7 @@
       </c>
       <c r="F338" s="7" t="inlineStr">
         <is>
-          <t>Ensemble de traductions de décisions judiciaires ukrainiennes relatives à la saisie conservatoire d'actions de MS : ordonnance du tribunal de district Shevchenkivsky en date du 07/09/2017 portant saisie de 207 592 actions inscrites au compte de Likaton Enterprises Limited et de 104 107 actions de Wang Xinlei auprès d'OTP Bank, énonçant la thèse de l'accusation relative à l'acquisition par la partie chinoise de 56,009 % des titres de MS et au défaut d'autorisation de l'AMKU (Comité anti-monopole d'Ukraine).</t>
+          <t>Ensemble de traductions de décisions judiciaires ukrainiennes relatives à la saisie conservatoire d'actions de MS : ordonnance du tribunal de district Shevchenkivsky en date du 7 septembre 2017 portant saisie de 207 592 actions inscrites au compte de Likaton Enterprises Limited et de 104 107 actions de Wang Xinlei auprès d'OTP Bank, énonçant la thèse de l'accusation relative à l'acquisition par la partie chinoise de 56,009 % des titres de MS et au défaut d'autorisation de l'AMKU (Comité anti-monopole d'Ukraine).</t>
         </is>
       </c>
     </row>
@@ -10435,12 +10435,12 @@
       </c>
       <c r="E339" s="7" t="inlineStr">
         <is>
-          <t>Granum Corporation ; Skyrizon ; Business House Helena ; Enfields ; Waldo ; Likaton ; Wang Xinlei ; Dragon Capital ; OTP Bank ; saisie d'actions ; 20/04/2018 ; 30/06/2021</t>
+          <t>Granum Corporation ; Skyrizon ; Business House Helena ; Enfields ; Waldo ; Likaton ; Wang Xinlei ; Dragon Capital ; OTP Bank ; saisie d'actions ; 20 avril 2018 ; 30 juin 2021</t>
         </is>
       </c>
       <c r="F339" s="7" t="inlineStr">
         <is>
-          <t>Dossier d'ordonnances judiciaires portant saisie pénale des blocs d'actions de MS inscrits au nom de Skyrizon Aircraft Holdings, Business House Helena, Enfields, Waldo Trade, Granum Corporation, Likaton Enterprises et Wang Xinlei. Comprend l'ordonnance de saisie du 20/04/2018 et l'arrêt de la Cour d'appel de Kyiv du 30/06/2021 statuant sur l'appel de Granum Corporation : infirmation partielle pour irrégularités procédurales de la requête initiale, la Cour d'appel ayant toutefois rendu une nouvelle décision maintenant expressément la saisie pénale sur les titres de Granum.</t>
+          <t>Dossier d'ordonnances judiciaires portant saisie pénale des blocs d'actions de MS inscrits au nom de Skyrizon Aircraft Holdings, Business House Helena, Enfields, Waldo Trade, Granum Corporation, Likaton Enterprises et Wang Xinlei. Comprend l'ordonnance de saisie du 20 avril 2018 et l'arrêt de la Cour d'appel de Kyiv du 30 juin 2021 statuant sur l'appel de Granum Corporation : infirmation partielle pour irrégularités procédurales de la requête initiale, la Cour d'appel ayant toutefois rendu une nouvelle décision maintenant expressément la saisie pénale sur les titres de Granum.</t>
         </is>
       </c>
     </row>
@@ -10496,7 +10496,7 @@
       <c r="E341" s="7" t="n"/>
       <c r="F341" s="7" t="inlineStr">
         <is>
-          <t>Dossier de traductions des écritures d'appel formées par la société Business House Helena A.G. à l'encontre de l'ordonnance de saisie pénale d'actions de MS du 06/08/2020.</t>
+          <t>Dossier de traductions des écritures d'appel formées par la société Business House Helena A.G. à l'encontre de l'ordonnance de saisie pénale d'actions de MS du 6 août 2020.</t>
         </is>
       </c>
     </row>
@@ -10556,7 +10556,7 @@
       <c r="E343" s="7" t="n"/>
       <c r="F343" s="7" t="inlineStr">
         <is>
-          <t>Dossier de deux ordonnances judiciaires en rectification d'erreur matérielle rendues sur l'ordonnance de saisie pénale conservatoire du 19/03/2021 (comptes OTP Bank).</t>
+          <t>Dossier de deux ordonnances judiciaires en rectification d'erreur matérielle rendues sur l'ordonnance de saisie pénale conservatoire du 19 mars 2021 (comptes OTP Bank).</t>
         </is>
       </c>
     </row>
@@ -10583,12 +10583,12 @@
       </c>
       <c r="E344" s="7" t="inlineStr">
         <is>
-          <t>Revenus de capitaux mobiliers ; cession d'actions ; VAB ; PwC ; Motor Dealer ; agent fiscal ; IRPP ; taxe militaire ; restitution du trop-perçu ; 14/02/2017</t>
+          <t>Revenus de capitaux mobiliers ; cession d'actions ; VAB ; PwC ; Motor Dealer ; agent fiscal ; IRPP ; taxe militaire ; restitution du trop-perçu ; 14 février 2017</t>
         </is>
       </c>
       <c r="F344" s="7" t="inlineStr">
         <is>
-          <t>Mémorandum fiscal du cabinet PwC du 14/02/2017 établi pour VAB relatif au régime fiscal des gains de cession de valeurs mobilières perçus par une personne physique en Ukraine consécutivement à la vente d'actions d'un émetteur ukrainien. Le document expose les règles d'assiette, le rôle d'agent fiscal de retenue dévolu à Motor Dealer, les modalités de paiement de l'impôt sur le revenu des personnes physiques (IRPP) et de la taxe militaire, ainsi que la restitution d'un trop-perçu fiscal au regard des justificatifs d'acquisition. PwC conclut sans ambiguïté que le circuit financier et fiscal mis en place respectait en lui-même la législation applicable.</t>
+          <t>Mémorandum fiscal du cabinet PwC du 14 février 2017 établi pour VAB relatif au régime fiscal des gains de cession de valeurs mobilières perçus par une personne physique en Ukraine consécutivement à la vente d'actions d'un émetteur ukrainien. Le document expose les règles d'assiette, le rôle d'agent fiscal de retenue dévolu à Motor Dealer, les modalités de paiement de l'impôt sur le revenu des personnes physiques (IRPP) et de la taxe militaire, ainsi que la restitution d'un trop-perçu fiscal au regard des justificatifs d'acquisition. PwC conclut sans ambiguïté que le circuit financier et fiscal mis en place respectait en lui-même la législation applicable.</t>
         </is>
       </c>
     </row>
@@ -10620,7 +10620,7 @@
       </c>
       <c r="F345" s="7" t="inlineStr">
         <is>
-          <t>Dossier documentaire comprenant des pièces bancaires, contractuelles, notariées et de publicité légale ukrainiennes. Le premier ensemble établit le crédit intervenu le 02/08/2016 sur les comptes de Vyacheslav Boguslayev (VAB) de deux virements totalisant 43 000 000 USD (14 362 000 USD en exécution de l'accord conclu avec Wang Xinlei et 28 638 000 USD au titre de la convention avec Likaton Enterprises, sous le libellé « Project Zoom II »). Le second volet a trait à l'acquisition par Boguslayev en 2021 de parts sociales de la SARL « Usine d'aviation de Vinnitsa » auprès de sociétés étrangères (Geoford LLP, Tabernus Corp., Aldon Business Inc. et Duncan Promotions Ltd.), avec production des actes de cession, des procès-verbaux de remise, des pièces de paiement, des actes notariés et des certificats d'enregistrement.</t>
+          <t>Dossier documentaire comprenant des pièces bancaires, contractuelles, notariées et de publicité légale ukrainiennes. Le premier ensemble établit le crédit intervenu le 2 août 2016 sur les comptes de Vyacheslav Boguslayev (VAB) de deux virements totalisant 43 000 000 USD (14 362 000 USD en exécution de l'accord conclu avec Wang Xinlei et 28 638 000 USD au titre de la convention avec Likaton Enterprises, sous le libellé « Project Zoom II »). Le second volet a trait à l'acquisition par Boguslayev en 2021 de parts sociales de la SARL « Usine d'aviation de Vinnitsa » auprès de sociétés étrangères (Geoford LLP, Tabernus Corp., Aldon Business Inc. et Duncan Promotions Ltd.), avec production des actes de cession, des procès-verbaux de remise, des pièces de paiement, des actes notariés et des certificats d'enregistrement.</t>
         </is>
       </c>
     </row>
@@ -10684,7 +10684,7 @@
       </c>
       <c r="F347" s="7" t="inlineStr">
         <is>
-          <t>Procès-verbal d'examen de données fiscales ukrainiennes traduites — versement complémentaire aux pièces du 21/01/2025.</t>
+          <t>Procès-verbal d'examen de données fiscales ukrainiennes traduites — versement complémentaire aux pièces du 21 janvier 2025.</t>
         </is>
       </c>
     </row>
@@ -11868,7 +11868,7 @@
       </c>
       <c r="F384" s="7" t="inlineStr">
         <is>
-          <t>Procès-verbal d'accès aux comptes bancaires monégasques d'AVB (Anton Vyacheslavovych Boguslayev).</t>
+          <t>Procès-verbal d'accès aux comptes bancaires monégasques d'AVB (Oleksandr Vyacheslavovych Boguslayev).</t>
         </is>
       </c>
     </row>
@@ -15154,7 +15154,7 @@
       </c>
       <c r="D490" s="7" t="inlineStr">
         <is>
-          <t>Résidence fiscale ; Fiscalité</t>
+          <t>Résidence ; Fiscalité</t>
         </is>
       </c>
       <c r="E490" s="7" t="inlineStr">
@@ -15164,7 +15164,7 @@
       </c>
       <c r="F490" s="7" t="inlineStr">
         <is>
-          <t>Facture de TLC Group du 04/02/2025 d'un montant de 18 000 EUR pour l'analyse des obligations d'AVB relatives au respect des critères de résidence à Monaco pour la période 2015–2024.</t>
+          <t>Facture de TLC Group du 4 février 2025 d'un montant de 18 000 EUR pour l'analyse des obligations d'AVB relatives au respect des critères de résidence à Monaco pour la période 2015–2024.</t>
         </is>
       </c>
     </row>
@@ -15186,7 +15186,7 @@
       </c>
       <c r="D491" s="7" t="inlineStr">
         <is>
-          <t>Résidence fiscale ; Fiscalité</t>
+          <t>Résidence ; Fiscalité</t>
         </is>
       </c>
       <c r="E491" s="7" t="inlineStr">

</xml_diff>